<commit_message>
added international aviation and changed library names in industry
</commit_message>
<xml_diff>
--- a/industry/industry_config.xlsx
+++ b/industry/industry_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fraunhofer-my.sharepoint.com/personal/rakesh_etikala_narendar_iee_fraunhofer_de/Documents/Desktop/sectoral-energy-demands/industry/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{32B99746-D61E-43DF-9653-52B59C7158BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FAD6AF4-4D8B-4C24-A81A-6BA76EF30A05}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{32B99746-D61E-43DF-9653-52B59C7158BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3115F34-CC2B-42F8-8F64-EFADADE3718B}"/>
   <bookViews>
-    <workbookView xWindow="7100" yWindow="2620" windowWidth="15330" windowHeight="11630" xr2:uid="{C5A233EC-3C33-42EA-837D-8F573F595C2A}"/>
+    <workbookView xWindow="2300" yWindow="2640" windowWidth="18630" windowHeight="15090" xr2:uid="{C5A233EC-3C33-42EA-837D-8F573F595C2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1029,9 +1029,6 @@
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
     </row>
     <row r="3" spans="1:63" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -1049,9 +1046,6 @@
       <c r="E3">
         <v>0</v>
       </c>
-      <c r="R3">
-        <v>5.8500000000000003E-2</v>
-      </c>
     </row>
     <row r="4" spans="1:63" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -1069,9 +1063,6 @@
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="R4">
-        <v>0.08</v>
-      </c>
     </row>
     <row r="5" spans="1:63" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -1089,9 +1080,6 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="R5">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" spans="1:63" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -1108,9 +1096,6 @@
       </c>
       <c r="E6">
         <v>0.01</v>
-      </c>
-      <c r="R6">
-        <v>5.8500000000000003E-2</v>
       </c>
     </row>
     <row r="7" spans="1:63" x14ac:dyDescent="0.35">

</xml_diff>